<commit_message>
Improve Alder pilot tasks
</commit_message>
<xml_diff>
--- a/companies/alder-ridge/source-files/Shared/Finance/Corporate Development/Active analyses/IC model inputs - 6.29 banker case.xlsx
+++ b/companies/alder-ridge/source-files/Shared/Finance/Corporate Development/Active analyses/IC model inputs - 6.29 banker case.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Checks" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QoE and Working Capital'!$A$4:$M$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QoE and Working Capital'!$A$4:$M$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Valuation'!$A$4:$M$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Transaction Models'!$A$4:$M$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Carveout and Integration'!$A$4:$M$44</definedName>
@@ -656,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -758,7 +758,7 @@
     <row r="5">
       <c r="A5" s="36" t="inlineStr">
         <is>
-          <t>DEV-00058</t>
+          <t>DEV-00059</t>
         </is>
       </c>
       <c r="B5" s="27" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="6">
       <c r="A6" s="36" t="inlineStr">
         <is>
-          <t>DEV-00059</t>
+          <t>DEV-00060</t>
         </is>
       </c>
       <c r="B6" s="27" t="inlineStr">
@@ -849,12 +849,12 @@
         </is>
       </c>
       <c r="H6" s="46" t="n">
-        <v>842293.92</v>
+        <v>842.2939200000001</v>
       </c>
       <c r="I6" s="27" t="inlineStr"/>
       <c r="J6" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K6" s="27" t="inlineStr">
@@ -872,7 +872,7 @@
     <row r="7">
       <c r="A7" s="36" t="inlineStr">
         <is>
-          <t>DEV-00060</t>
+          <t>DEV-00061</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
@@ -906,12 +906,12 @@
         </is>
       </c>
       <c r="H7" s="46" t="n">
-        <v>758.1</v>
+        <v>758100</v>
       </c>
       <c r="I7" s="27" t="inlineStr"/>
       <c r="J7" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K7" s="27" t="inlineStr">
@@ -929,7 +929,7 @@
     <row r="8">
       <c r="A8" s="36" t="inlineStr">
         <is>
-          <t>DEV-00061</t>
+          <t>DEV-00062</t>
         </is>
       </c>
       <c r="B8" s="27" t="inlineStr">
@@ -986,7 +986,7 @@
     <row r="9">
       <c r="A9" s="36" t="inlineStr">
         <is>
-          <t>DEV-00062</t>
+          <t>DEV-00063</t>
         </is>
       </c>
       <c r="B9" s="27" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="10">
       <c r="A10" s="36" t="inlineStr">
         <is>
-          <t>DEV-00063</t>
+          <t>DEV-00064</t>
         </is>
       </c>
       <c r="B10" s="27" t="inlineStr">
@@ -1077,12 +1077,12 @@
         </is>
       </c>
       <c r="H10" s="46" t="n">
-        <v>816900</v>
+        <v>816.9</v>
       </c>
       <c r="I10" s="27" t="inlineStr"/>
       <c r="J10" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K10" s="27" t="inlineStr">
@@ -1100,7 +1100,7 @@
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
         <is>
-          <t>DEV-00064</t>
+          <t>DEV-00065</t>
         </is>
       </c>
       <c r="B11" s="27" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Remaining risk register</t>
+          <t>QoE adjustment evidence</t>
         </is>
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>Top-customer concentration</t>
+          <t>Vacant CFO run-rate cost</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr">
@@ -1130,16 +1130,16 @@
       </c>
       <c r="G11" s="27" t="inlineStr">
         <is>
-          <t>EBITDA impact</t>
+          <t>Seller proposed EBITDA adjustment</t>
         </is>
       </c>
       <c r="H11" s="46" t="n">
-        <v>1236</v>
+        <v>0</v>
       </c>
       <c r="I11" s="27" t="inlineStr"/>
       <c r="J11" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K11" s="27" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
         <is>
-          <t>DEV-00065</t>
+          <t>DEV-00066</t>
         </is>
       </c>
       <c r="B12" s="27" t="inlineStr">
@@ -1167,17 +1167,17 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Redwood monthly P&amp;L</t>
+          <t>Remaining risk register</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Top-customer concentration</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>Diligence</t>
         </is>
       </c>
       <c r="F12" s="27" t="inlineStr">
@@ -1187,16 +1187,16 @@
       </c>
       <c r="G12" s="27" t="inlineStr">
         <is>
-          <t>Operating expense before D&amp;A</t>
+          <t>Probability</t>
         </is>
       </c>
       <c r="H12" s="46" t="n">
-        <v>717600</v>
+        <v>0.8320000000000001</v>
       </c>
       <c r="I12" s="27" t="inlineStr"/>
       <c r="J12" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K12" s="27" t="inlineStr">
@@ -1214,7 +1214,7 @@
     <row r="13">
       <c r="A13" s="36" t="inlineStr">
         <is>
-          <t>DEV-00066</t>
+          <t>DEV-00067</t>
         </is>
       </c>
       <c r="B13" s="27" t="inlineStr">
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="H13" s="46" t="n">
-        <v>2494800</v>
+        <v>2362500</v>
       </c>
       <c r="I13" s="27" t="inlineStr"/>
       <c r="J13" s="27" t="inlineStr">
@@ -1271,7 +1271,7 @@
     <row r="14">
       <c r="A14" s="36" t="inlineStr">
         <is>
-          <t>DEV-00067</t>
+          <t>DEV-00068</t>
         </is>
       </c>
       <c r="B14" s="27" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="F14" s="27" t="inlineStr">
@@ -1305,12 +1305,12 @@
         </is>
       </c>
       <c r="H14" s="46" t="n">
-        <v>879228.5999999999</v>
+        <v>834.1949400000001</v>
       </c>
       <c r="I14" s="27" t="inlineStr"/>
       <c r="J14" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K14" s="27" t="inlineStr">
@@ -1328,7 +1328,7 @@
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>DEV-00068</t>
+          <t>DEV-00069</t>
         </is>
       </c>
       <c r="B15" s="27" t="inlineStr">
@@ -1362,12 +1362,12 @@
         </is>
       </c>
       <c r="H15" s="46" t="n">
-        <v>775.84</v>
+        <v>750880</v>
       </c>
       <c r="I15" s="27" t="inlineStr"/>
       <c r="J15" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K15" s="27" t="inlineStr">
@@ -1385,41 +1385,41 @@
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>DEV-00069</t>
+          <t>DEV-00148</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Redwood Controls quality-of-earnings normalization</t>
+          <t>BluePeak normalized working-capital peg</t>
         </is>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Redwood monthly P&amp;L</t>
+          <t>Historical normalized NWC</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>BluePeak</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F16" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G16" s="27" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Trade AR</t>
         </is>
       </c>
       <c r="H16" s="46" t="n">
-        <v>2803500</v>
+        <v>4171500</v>
       </c>
       <c r="I16" s="27" t="inlineStr"/>
       <c r="J16" s="27" t="inlineStr">
@@ -1442,7 +1442,7 @@
     <row r="17">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>DEV-00148</t>
+          <t>DEV-00149</t>
         </is>
       </c>
       <c r="B17" s="27" t="inlineStr">
@@ -1462,26 +1462,26 @@
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="F17" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
         <is>
-          <t>Trade AR</t>
+          <t>Trade AP</t>
         </is>
       </c>
       <c r="H17" s="46" t="n">
-        <v>4171500</v>
+        <v>2137.2</v>
       </c>
       <c r="I17" s="27" t="inlineStr"/>
       <c r="J17" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K17" s="27" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="18">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>DEV-00149</t>
+          <t>DEV-00150</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -1519,26 +1519,26 @@
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F18" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G18" s="27" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Deferred revenue</t>
         </is>
       </c>
       <c r="H18" s="46" t="n">
-        <v>1214.72</v>
+        <v>312900</v>
       </c>
       <c r="I18" s="27" t="inlineStr"/>
       <c r="J18" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K18" s="27" t="inlineStr">
@@ -1556,7 +1556,7 @@
     <row r="19">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>DEV-00150</t>
+          <t>DEV-00151</t>
         </is>
       </c>
       <c r="B19" s="27" t="inlineStr">
@@ -1576,21 +1576,21 @@
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F19" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G19" s="27" t="inlineStr">
         <is>
-          <t>Trade AP</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="H19" s="46" t="n">
-        <v>2194500</v>
+        <v>1258660</v>
       </c>
       <c r="I19" s="27" t="inlineStr"/>
       <c r="J19" s="27" t="inlineStr">
@@ -1613,7 +1613,7 @@
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>DEV-00151</t>
+          <t>DEV-00152</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F20" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G20" s="27" t="inlineStr">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="H20" s="46" t="n">
-        <v>458350</v>
+        <v>473200</v>
       </c>
       <c r="I20" s="27" t="inlineStr"/>
       <c r="J20" s="27" t="inlineStr">
@@ -1670,7 +1670,7 @@
     <row r="21">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>DEV-00152</t>
+          <t>DEV-00153</t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
@@ -1690,26 +1690,26 @@
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="F21" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G21" s="27" t="inlineStr">
         <is>
-          <t>Deferred revenue</t>
+          <t>Trade AR</t>
         </is>
       </c>
       <c r="H21" s="46" t="n">
-        <v>318240</v>
+        <v>4656.75</v>
       </c>
       <c r="I21" s="27" t="inlineStr"/>
       <c r="J21" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K21" s="27" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="22">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t>DEV-00153</t>
+          <t>DEV-00154</t>
         </is>
       </c>
       <c r="B22" s="27" t="inlineStr">
@@ -1747,26 +1747,26 @@
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F22" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G22" s="27" t="inlineStr">
         <is>
-          <t>Include in peg</t>
+          <t>Trade AP</t>
         </is>
       </c>
       <c r="H22" s="46" t="n">
-        <v>0</v>
+        <v>2369000</v>
       </c>
       <c r="I22" s="27" t="inlineStr"/>
       <c r="J22" s="27" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K22" s="27" t="inlineStr">
@@ -1784,7 +1784,7 @@
     <row r="23">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>DEV-00154</t>
+          <t>DEV-00155</t>
         </is>
       </c>
       <c r="B23" s="27" t="inlineStr">
@@ -1804,21 +1804,21 @@
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="F23" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G23" s="27" t="inlineStr">
         <is>
-          <t>Trade AR</t>
+          <t>Deferred revenue</t>
         </is>
       </c>
       <c r="H23" s="46" t="n">
-        <v>4568050</v>
+        <v>339040</v>
       </c>
       <c r="I23" s="27" t="inlineStr"/>
       <c r="J23" s="27" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t>DEV-00155</t>
+          <t>DEV-00156</t>
         </is>
       </c>
       <c r="B24" s="27" t="inlineStr">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E24" s="27" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F24" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G24" s="27" t="inlineStr">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="H24" s="46" t="n">
-        <v>1345760</v>
+        <v>1415400</v>
       </c>
       <c r="I24" s="27" t="inlineStr"/>
       <c r="J24" s="27" t="inlineStr">
@@ -1898,7 +1898,7 @@
     <row r="25">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>DEV-00156</t>
+          <t>DEV-00157</t>
         </is>
       </c>
       <c r="B25" s="27" t="inlineStr">
@@ -1908,36 +1908,36 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>Historical normalized NWC</t>
+          <t>Estimated closing balance sheet</t>
         </is>
       </c>
       <c r="D25" s="27" t="inlineStr">
         <is>
-          <t>BluePeak</t>
+          <t>Payroll and benefits accrual</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>Estimated closing</t>
         </is>
       </c>
       <c r="F25" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G25" s="27" t="inlineStr">
         <is>
-          <t>Trade AP</t>
+          <t>Balance</t>
         </is>
       </c>
       <c r="H25" s="46" t="n">
-        <v>2451750</v>
+        <v>319.3</v>
       </c>
       <c r="I25" s="27" t="inlineStr"/>
       <c r="J25" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K25" s="27" t="inlineStr">
@@ -1955,41 +1955,41 @@
     <row r="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>DEV-00157</t>
+          <t>DEV-00460</t>
         </is>
       </c>
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>BluePeak normalized working-capital peg</t>
+          <t>Create the Pioneer QoE and purchase-price bridge</t>
         </is>
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Historical normalized NWC</t>
+          <t>Target reported results</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>BluePeak</t>
+          <t>Pioneer HVAC</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F26" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G26" s="27" t="inlineStr">
         <is>
-          <t>Accrued operating liabilities</t>
+          <t>Reported EBITDA</t>
         </is>
       </c>
       <c r="H26" s="46" t="n">
-        <v>494.4</v>
+        <v>5005.8</v>
       </c>
       <c r="I26" s="27" t="inlineStr"/>
       <c r="J26" s="27" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>DEV-00460</t>
+          <t>DEV-00461</t>
         </is>
       </c>
       <c r="B27" s="27" t="inlineStr">
@@ -2022,36 +2022,36 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Target reported results</t>
+          <t>QoE adjustments</t>
         </is>
       </c>
       <c r="D27" s="27" t="inlineStr">
         <is>
-          <t>Pioneer HVAC</t>
+          <t>Proposed procurement synergy</t>
         </is>
       </c>
       <c r="E27" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>LTM 2026-06-30</t>
         </is>
       </c>
       <c r="F27" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G27" s="27" t="inlineStr">
         <is>
-          <t>Reported EBITDA</t>
+          <t>EBITDA adjustment</t>
         </is>
       </c>
       <c r="H27" s="46" t="n">
-        <v>5005.8</v>
+        <v>634400</v>
       </c>
       <c r="I27" s="27" t="inlineStr"/>
       <c r="J27" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K27" s="27" t="inlineStr">
@@ -2069,7 +2069,7 @@
     <row r="28">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>DEV-00461</t>
+          <t>DEV-00462</t>
         </is>
       </c>
       <c r="B28" s="27" t="inlineStr">
@@ -2079,31 +2079,31 @@
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>QoE adjustments</t>
+          <t>Target monthly working capital</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>Proposed procurement synergy</t>
+          <t>Pioneer HVAC</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>LTM 2026-06-30</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F28" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G28" s="27" t="inlineStr">
         <is>
-          <t>EBITDA adjustment</t>
+          <t>Accounts receivable</t>
         </is>
       </c>
       <c r="H28" s="46" t="n">
-        <v>634400</v>
+        <v>2152500</v>
       </c>
       <c r="I28" s="27" t="inlineStr"/>
       <c r="J28" s="27" t="inlineStr">
@@ -2126,7 +2126,7 @@
     <row r="29">
       <c r="A29" s="36" t="inlineStr">
         <is>
-          <t>DEV-00462</t>
+          <t>DEV-00463</t>
         </is>
       </c>
       <c r="B29" s="27" t="inlineStr">
@@ -2146,21 +2146,21 @@
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="F29" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G29" s="27" t="inlineStr">
         <is>
-          <t>Accounts receivable</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="H29" s="46" t="n">
-        <v>2152500</v>
+        <v>7055500</v>
       </c>
       <c r="I29" s="27" t="inlineStr"/>
       <c r="J29" s="27" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="30">
       <c r="A30" s="36" t="inlineStr">
         <is>
-          <t>DEV-00463</t>
+          <t>DEV-00464</t>
         </is>
       </c>
       <c r="B30" s="27" t="inlineStr">
@@ -2203,26 +2203,26 @@
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F30" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G30" s="27" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Accounts payable</t>
         </is>
       </c>
       <c r="H30" s="46" t="n">
-        <v>7055500</v>
+        <v>1341.6</v>
       </c>
       <c r="I30" s="27" t="inlineStr"/>
       <c r="J30" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K30" s="27" t="inlineStr">
@@ -2240,7 +2240,7 @@
     <row r="31">
       <c r="A31" s="36" t="inlineStr">
         <is>
-          <t>DEV-00464</t>
+          <t>DEV-00465</t>
         </is>
       </c>
       <c r="B31" s="27" t="inlineStr">
@@ -2260,26 +2260,26 @@
       </c>
       <c r="E31" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F31" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G31" s="27" t="inlineStr">
         <is>
-          <t>Accounts payable</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="H31" s="46" t="n">
-        <v>1341.6</v>
+        <v>3055500</v>
       </c>
       <c r="I31" s="27" t="inlineStr"/>
       <c r="J31" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K31" s="27" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="32">
       <c r="A32" s="36" t="inlineStr">
         <is>
-          <t>DEV-00465</t>
+          <t>DEV-00466</t>
         </is>
       </c>
       <c r="B32" s="27" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Target monthly working capital</t>
+          <t>Purchase price terms</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
@@ -2317,21 +2317,21 @@
       </c>
       <c r="E32" s="27" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F32" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G32" s="27" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Seller retained tax receivable</t>
         </is>
       </c>
       <c r="H32" s="46" t="n">
-        <v>3055500</v>
+        <v>247200</v>
       </c>
       <c r="I32" s="27" t="inlineStr"/>
       <c r="J32" s="27" t="inlineStr">
@@ -2354,7 +2354,7 @@
     <row r="33">
       <c r="A33" s="36" t="inlineStr">
         <is>
-          <t>DEV-00466</t>
+          <t>DEV-00467</t>
         </is>
       </c>
       <c r="B33" s="27" t="inlineStr">
@@ -2364,36 +2364,36 @@
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Purchase price terms</t>
+          <t>QoE adjustments</t>
         </is>
       </c>
       <c r="D33" s="27" t="inlineStr">
         <is>
-          <t>Pioneer HVAC</t>
+          <t>Uninsured storm loss</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>LTM 2026-06-30</t>
         </is>
       </c>
       <c r="F33" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G33" s="27" t="inlineStr">
         <is>
-          <t>Seller retained tax receivable</t>
+          <t>Include in QoE</t>
         </is>
       </c>
       <c r="H33" s="46" t="n">
-        <v>247200</v>
+        <v>1.04</v>
       </c>
       <c r="I33" s="27" t="inlineStr"/>
       <c r="J33" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="K33" s="27" t="inlineStr">
@@ -2411,7 +2411,7 @@
     <row r="34">
       <c r="A34" s="36" t="inlineStr">
         <is>
-          <t>DEV-00467</t>
+          <t>DEV-00468</t>
         </is>
       </c>
       <c r="B34" s="27" t="inlineStr">
@@ -2426,31 +2426,31 @@
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>Uninsured storm loss</t>
+          <t>Banker revenue uplift</t>
         </is>
       </c>
       <c r="E34" s="27" t="inlineStr">
         <is>
-          <t>LTM 2026-06-30</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F34" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G34" s="27" t="inlineStr">
         <is>
-          <t>Include in QoE</t>
+          <t>EBITDA adjustment</t>
         </is>
       </c>
       <c r="H34" s="46" t="n">
-        <v>1.04</v>
+        <v>567</v>
       </c>
       <c r="I34" s="27" t="inlineStr"/>
       <c r="J34" s="27" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K34" s="27" t="inlineStr">
@@ -2468,7 +2468,7 @@
     <row r="35">
       <c r="A35" s="36" t="inlineStr">
         <is>
-          <t>DEV-00468</t>
+          <t>DEV-00469</t>
         </is>
       </c>
       <c r="B35" s="27" t="inlineStr">
@@ -2478,36 +2478,36 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>QoE adjustments</t>
+          <t>Target monthly working capital</t>
         </is>
       </c>
       <c r="D35" s="27" t="inlineStr">
         <is>
-          <t>Banker revenue uplift</t>
+          <t>Pioneer HVAC</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="F35" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G35" s="27" t="inlineStr">
         <is>
-          <t>EBITDA adjustment</t>
+          <t>Accounts receivable</t>
         </is>
       </c>
       <c r="H35" s="46" t="n">
-        <v>567</v>
+        <v>2276300</v>
       </c>
       <c r="I35" s="27" t="inlineStr"/>
       <c r="J35" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K35" s="27" t="inlineStr">
@@ -2525,7 +2525,7 @@
     <row r="36">
       <c r="A36" s="36" t="inlineStr">
         <is>
-          <t>DEV-00469</t>
+          <t>DEV-00470</t>
         </is>
       </c>
       <c r="B36" s="27" t="inlineStr">
@@ -2545,21 +2545,21 @@
       </c>
       <c r="E36" s="27" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F36" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G36" s="27" t="inlineStr">
         <is>
-          <t>Accounts receivable</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="H36" s="46" t="n">
-        <v>2276300</v>
+        <v>7030400</v>
       </c>
       <c r="I36" s="27" t="inlineStr"/>
       <c r="J36" s="27" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="37">
       <c r="A37" s="36" t="inlineStr">
         <is>
-          <t>DEV-00470</t>
+          <t>DEV-00471</t>
         </is>
       </c>
       <c r="B37" s="27" t="inlineStr">
@@ -2602,21 +2602,21 @@
       </c>
       <c r="E37" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F37" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G37" s="27" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Accounts payable</t>
         </is>
       </c>
       <c r="H37" s="46" t="n">
-        <v>7030400</v>
+        <v>1396500</v>
       </c>
       <c r="I37" s="27" t="inlineStr"/>
       <c r="J37" s="27" t="inlineStr">
@@ -2639,7 +2639,7 @@
     <row r="38">
       <c r="A38" s="36" t="inlineStr">
         <is>
-          <t>DEV-00471</t>
+          <t>DEV-00472</t>
         </is>
       </c>
       <c r="B38" s="27" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>Target monthly working capital</t>
+          <t>Purchase price terms</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
@@ -2659,26 +2659,26 @@
       </c>
       <c r="E38" s="27" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F38" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G38" s="27" t="inlineStr">
         <is>
-          <t>Accounts payable</t>
+          <t>Funded debt</t>
         </is>
       </c>
       <c r="H38" s="46" t="n">
-        <v>1396500</v>
+        <v>4841</v>
       </c>
       <c r="I38" s="27" t="inlineStr"/>
       <c r="J38" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K38" s="27" t="inlineStr">
@@ -2696,7 +2696,7 @@
     <row r="39">
       <c r="A39" s="36" t="inlineStr">
         <is>
-          <t>DEV-00472</t>
+          <t>DEV-00473</t>
         </is>
       </c>
       <c r="B39" s="27" t="inlineStr">
@@ -2706,36 +2706,36 @@
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Purchase price terms</t>
+          <t>QoE adjustments</t>
         </is>
       </c>
       <c r="D39" s="27" t="inlineStr">
         <is>
-          <t>Pioneer HVAC</t>
+          <t>Owner compensation normalization</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>LTM 2026-06-30</t>
         </is>
       </c>
       <c r="F39" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G39" s="27" t="inlineStr">
         <is>
-          <t>Funded debt</t>
+          <t>EBITDA adjustment</t>
         </is>
       </c>
       <c r="H39" s="46" t="n">
-        <v>4841</v>
+        <v>436800</v>
       </c>
       <c r="I39" s="27" t="inlineStr"/>
       <c r="J39" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K39" s="27" t="inlineStr">
@@ -2753,7 +2753,7 @@
     <row r="40">
       <c r="A40" s="36" t="inlineStr">
         <is>
-          <t>DEV-00473</t>
+          <t>DEV-00474</t>
         </is>
       </c>
       <c r="B40" s="27" t="inlineStr">
@@ -2768,31 +2768,31 @@
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>Owner compensation normalization</t>
+          <t>Proposed procurement synergy</t>
         </is>
       </c>
       <c r="E40" s="27" t="inlineStr">
         <is>
-          <t>LTM 2026-06-30</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F40" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G40" s="27" t="inlineStr">
         <is>
-          <t>EBITDA adjustment</t>
+          <t>Include in QoE</t>
         </is>
       </c>
       <c r="H40" s="46" t="n">
-        <v>436800</v>
+        <v>0</v>
       </c>
       <c r="I40" s="27" t="inlineStr"/>
       <c r="J40" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="K40" s="27" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="41">
       <c r="A41" s="36" t="inlineStr">
         <is>
-          <t>DEV-00474</t>
+          <t>DEV-00475</t>
         </is>
       </c>
       <c r="B41" s="27" t="inlineStr">
@@ -2820,36 +2820,36 @@
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>QoE adjustments</t>
+          <t>Target monthly working capital</t>
         </is>
       </c>
       <c r="D41" s="27" t="inlineStr">
         <is>
-          <t>Proposed procurement synergy</t>
+          <t>Pioneer HVAC</t>
         </is>
       </c>
       <c r="E41" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="F41" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G41" s="27" t="inlineStr">
         <is>
-          <t>Include in QoE</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="H41" s="46" t="n">
-        <v>0</v>
+        <v>2492600</v>
       </c>
       <c r="I41" s="27" t="inlineStr"/>
       <c r="J41" s="27" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K41" s="27" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="42">
       <c r="A42" s="36" t="inlineStr">
         <is>
-          <t>DEV-00475</t>
+          <t>DEV-00489</t>
         </is>
       </c>
       <c r="B42" s="27" t="inlineStr">
@@ -2877,31 +2877,31 @@
       </c>
       <c r="C42" s="27" t="inlineStr">
         <is>
-          <t>Target monthly working capital</t>
+          <t>Locked box leakage review</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>Pioneer HVAC</t>
+          <t>Owner dividend</t>
         </is>
       </c>
       <c r="E42" s="27" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F42" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G42" s="27" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Cash outflow</t>
         </is>
       </c>
       <c r="H42" s="46" t="n">
-        <v>2492600</v>
+        <v>319300</v>
       </c>
       <c r="I42" s="27" t="inlineStr"/>
       <c r="J42" s="27" t="inlineStr">
@@ -2924,7 +2924,7 @@
     <row r="43">
       <c r="A43" s="36" t="inlineStr">
         <is>
-          <t>DEV-00489</t>
+          <t>DEV-00490</t>
         </is>
       </c>
       <c r="B43" s="27" t="inlineStr">
@@ -2939,31 +2939,31 @@
       </c>
       <c r="D43" s="27" t="inlineStr">
         <is>
-          <t>Owner dividend</t>
+          <t>Ordinary payroll</t>
         </is>
       </c>
       <c r="E43" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>Signing to close</t>
         </is>
       </c>
       <c r="F43" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G43" s="27" t="inlineStr">
         <is>
-          <t>Cash outflow</t>
+          <t>Permitted leakage</t>
         </is>
       </c>
       <c r="H43" s="46" t="n">
-        <v>319300</v>
+        <v>1.04</v>
       </c>
       <c r="I43" s="27" t="inlineStr"/>
       <c r="J43" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="K43" s="27" t="inlineStr">
@@ -2981,7 +2981,7 @@
     <row r="44">
       <c r="A44" s="36" t="inlineStr">
         <is>
-          <t>DEV-00490</t>
+          <t>DEV-00491</t>
         </is>
       </c>
       <c r="B44" s="27" t="inlineStr">
@@ -2996,17 +2996,17 @@
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>Ordinary payroll</t>
+          <t>Owner dividend</t>
         </is>
       </c>
       <c r="E44" s="27" t="inlineStr">
         <is>
-          <t>Signing to close</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F44" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G44" s="27" t="inlineStr">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="H44" s="46" t="n">
-        <v>1.04</v>
+        <v>0</v>
       </c>
       <c r="I44" s="27" t="inlineStr"/>
       <c r="J44" s="27" t="inlineStr">
@@ -3038,7 +3038,7 @@
     <row r="45">
       <c r="A45" s="36" t="inlineStr">
         <is>
-          <t>DEV-00491</t>
+          <t>DEV-00492</t>
         </is>
       </c>
       <c r="B45" s="27" t="inlineStr">
@@ -3048,36 +3048,36 @@
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>Locked box leakage review</t>
+          <t>Closing funds flow terms</t>
         </is>
       </c>
       <c r="D45" s="27" t="inlineStr">
         <is>
-          <t>Owner dividend</t>
+          <t>Pioneer HVAC</t>
         </is>
       </c>
       <c r="E45" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="F45" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G45" s="27" t="inlineStr">
         <is>
-          <t>Permitted leakage</t>
+          <t>Escrow percent of adjusted equity price</t>
         </is>
       </c>
       <c r="H45" s="46" t="n">
-        <v>0</v>
+        <v>0.07725</v>
       </c>
       <c r="I45" s="27" t="inlineStr"/>
       <c r="J45" s="27" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K45" s="27" t="inlineStr">
@@ -3095,7 +3095,7 @@
     <row r="46">
       <c r="A46" s="36" t="inlineStr">
         <is>
-          <t>DEV-00492</t>
+          <t>DEV-00493</t>
         </is>
       </c>
       <c r="B46" s="27" t="inlineStr">
@@ -3105,36 +3105,36 @@
       </c>
       <c r="C46" s="27" t="inlineStr">
         <is>
-          <t>Closing funds flow terms</t>
+          <t>Locked box leakage review</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>Pioneer HVAC</t>
+          <t>Tax distribution</t>
         </is>
       </c>
       <c r="E46" s="27" t="inlineStr">
         <is>
-          <t>Closing</t>
+          <t>2026-05 working copy</t>
         </is>
       </c>
       <c r="F46" s="27" t="inlineStr">
         <is>
-          <t>Management stretch</t>
+          <t>Approved case</t>
         </is>
       </c>
       <c r="G46" s="27" t="inlineStr">
         <is>
-          <t>Escrow percent of adjusted equity price</t>
+          <t>Cash outflow</t>
         </is>
       </c>
       <c r="H46" s="46" t="n">
-        <v>0.07725</v>
+        <v>192400</v>
       </c>
       <c r="I46" s="27" t="inlineStr"/>
       <c r="J46" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K46" s="27" t="inlineStr">
@@ -3152,7 +3152,7 @@
     <row r="47">
       <c r="A47" s="36" t="inlineStr">
         <is>
-          <t>DEV-00493</t>
+          <t>DEV-00494</t>
         </is>
       </c>
       <c r="B47" s="27" t="inlineStr">
@@ -3162,31 +3162,31 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Locked box leakage review</t>
+          <t>Closing funds flow terms</t>
         </is>
       </c>
       <c r="D47" s="27" t="inlineStr">
         <is>
-          <t>Tax distribution</t>
+          <t>Pioneer HVAC</t>
         </is>
       </c>
       <c r="E47" s="27" t="inlineStr">
         <is>
-          <t>2026-05 working copy</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="F47" s="27" t="inlineStr">
         <is>
-          <t>Approved case</t>
+          <t>Management stretch</t>
         </is>
       </c>
       <c r="G47" s="27" t="inlineStr">
         <is>
-          <t>Cash outflow</t>
+          <t>Earnout face value</t>
         </is>
       </c>
       <c r="H47" s="46" t="n">
-        <v>192400</v>
+        <v>4725000</v>
       </c>
       <c r="I47" s="27" t="inlineStr"/>
       <c r="J47" s="27" t="inlineStr">
@@ -3206,65 +3206,8 @@
       </c>
       <c r="M47" s="27" t="inlineStr"/>
     </row>
-    <row r="48">
-      <c r="A48" s="36" t="inlineStr">
-        <is>
-          <t>DEV-00494</t>
-        </is>
-      </c>
-      <c r="B48" s="27" t="inlineStr">
-        <is>
-          <t>Create the Pioneer QoE and purchase-price bridge</t>
-        </is>
-      </c>
-      <c r="C48" s="27" t="inlineStr">
-        <is>
-          <t>Closing funds flow terms</t>
-        </is>
-      </c>
-      <c r="D48" s="27" t="inlineStr">
-        <is>
-          <t>Pioneer HVAC</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr">
-        <is>
-          <t>Closing</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="inlineStr">
-        <is>
-          <t>Management stretch</t>
-        </is>
-      </c>
-      <c r="G48" s="27" t="inlineStr">
-        <is>
-          <t>Earnout face value</t>
-        </is>
-      </c>
-      <c r="H48" s="46" t="n">
-        <v>4725000</v>
-      </c>
-      <c r="I48" s="27" t="inlineStr"/>
-      <c r="J48" s="27" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="K48" s="27" t="inlineStr">
-        <is>
-          <t>Earlier management working export</t>
-        </is>
-      </c>
-      <c r="L48" s="47" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="M48" s="27" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M48"/>
+  <autoFilter ref="A4:M47"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
@@ -13150,10 +13093,10 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="40">
-        <f>COUNTA('QoE and Working Capital'!$A$5:$A$48)</f>
+        <f>COUNTA('QoE and Working Capital'!$A$5:$A$47)</f>
         <v/>
       </c>
       <c r="D5" s="40">

</xml_diff>